<commit_message>
done with gz dzt
</commit_message>
<xml_diff>
--- a/mode_docx_gen/1.xlsx
+++ b/mode_docx_gen/1.xlsx
@@ -435,353 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="20" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_hvptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_ptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_ptoc2_tovctoc</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_ptoc1_lvarctoc</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_ptoc1_ltcblktoc</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_hvptoc1_strpalc</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_lvptoc1_strpalc</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_lvptoc2_strpalc</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_hvptoc1_tpalc</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_lvptoc1_tpalc</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_lvptoc2_tpalc</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_lvoileqpalc_eqpalc</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>SGF2_lvoileqpalc_eqpalc</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>SGF3_lvoileqpalc_eqpalc</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_ptrc1_tprmofflvlgc</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_rbre1_tprmofflvlgc</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Номинальный ток входа ВН</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Номинальный ток входа НН1</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Номинальный ток входа НН2</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="P2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q2" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="R2" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="S2" s="2" t="n">
-        <v>5</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:O2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>T1_hvptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_hvptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>T1_ptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_ptoc1_tovctoc</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>T1_ptoc2_tovctoc</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_ptoc2_tovctoc</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_ptoc1_lvarctoc</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_ptoc1_ltcblktoc</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_hvptoc1_strpalc</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_lvptoc1_strpalc</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_lvptoc2_strpalc</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_hvptoc1_tpalc</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_lvptoc1_tpalc</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Iset_lvptoc2_tpalc</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>T1_lvoileqpalc_eqpalc</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="J2" s="2" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="K2" s="2" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="L2" s="2" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="M2" s="2" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="N2" s="2" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="O2" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AC2"/>
+  <dimension ref="A1:AQ2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -813,152 +467,759 @@
     <col width="20" customWidth="1" min="27" max="27"/>
     <col width="20" customWidth="1" min="28" max="28"/>
     <col width="20" customWidth="1" min="29" max="29"/>
+    <col width="20" customWidth="1" min="30" max="30"/>
+    <col width="20" customWidth="1" min="31" max="31"/>
+    <col width="20" customWidth="1" min="32" max="32"/>
+    <col width="20" customWidth="1" min="33" max="33"/>
+    <col width="20" customWidth="1" min="34" max="34"/>
+    <col width="20" customWidth="1" min="35" max="35"/>
+    <col width="20" customWidth="1" min="36" max="36"/>
+    <col width="20" customWidth="1" min="37" max="37"/>
+    <col width="20" customWidth="1" min="38" max="38"/>
+    <col width="20" customWidth="1" min="39" max="39"/>
+    <col width="20" customWidth="1" min="40" max="40"/>
+    <col width="20" customWidth="1" min="41" max="41"/>
+    <col width="20" customWidth="1" min="42" max="42"/>
+    <col width="20" customWidth="1" min="43" max="43"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>IA</t>
+          <t>SGF1_oilptrc1_apttechlgc</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>IB</t>
+          <t>SGF2_oilptrc1_apttechlgc</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>IC</t>
+          <t>SGF1_winptrc1_apttechlgc</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>IA1</t>
+          <t>SGF2_winptrc1_apttechlgc</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>IB1</t>
+          <t>SGF1_vlvptrc1_apttechlgc</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>IC1</t>
+          <t>SGF2_vlvptrc1_apttechlgc</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>SGF1_prvlvptrc1_almtechlgc</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>SGF1_shvlvptrc1_almtechlgc</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>SGF1_levptrc1_almtechlgc</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>SGF1_ptrc1_talmgaslgc</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>SGF2_ptrc1_talmgaslgc</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>SGF1_ptrc1_ttrgaslgc</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>SGF2_ptrc1_ttrgaslgc</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>SGF1_ptrc1_tltcgaslgc</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>SGF2_ptrc1_tltcgaslgc</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>SGF1_ptrc1_tprmofflvlgc</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>SGF1_rbre1_tprmofflvlgc</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>SGF1_lvalh</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>SGF2_lvalh</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>SGF3_lvalh</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>SGF4_lvalh</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>SGF5_lvalh</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>SGF6_lvalh</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>SGF7_lvalh</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>SGF8_lvalh</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>SGF9_lvalh</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>SGF10_lvalh</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>SGF11_lvalh</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>SGF12_lvalh</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>SGF13_lvalh</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>SGF1_tsa</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>SGF2_tsa</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>SGF3_tsa</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>SGF4_tsa</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>SGF5_tsa</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>SGF6_tsa</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>SGF7_tsa</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>SGF8_tsa</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>SGF9_tsa</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>SGF10_tsa</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>SGF11_tsa</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>SGF12_tsa</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>SGF13_tsa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>T1_apttechlgc</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>T1_ptrc1_talmgaslgc</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>T1_ttrgaslgc</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>T1_tltcgaslgc</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:BA2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="20" customWidth="1" min="28" max="28"/>
+    <col width="20" customWidth="1" min="29" max="29"/>
+    <col width="20" customWidth="1" min="30" max="30"/>
+    <col width="20" customWidth="1" min="31" max="31"/>
+    <col width="20" customWidth="1" min="32" max="32"/>
+    <col width="20" customWidth="1" min="33" max="33"/>
+    <col width="20" customWidth="1" min="34" max="34"/>
+    <col width="20" customWidth="1" min="35" max="35"/>
+    <col width="20" customWidth="1" min="36" max="36"/>
+    <col width="20" customWidth="1" min="37" max="37"/>
+    <col width="20" customWidth="1" min="38" max="38"/>
+    <col width="20" customWidth="1" min="39" max="39"/>
+    <col width="20" customWidth="1" min="40" max="40"/>
+    <col width="20" customWidth="1" min="41" max="41"/>
+    <col width="20" customWidth="1" min="42" max="42"/>
+    <col width="20" customWidth="1" min="43" max="43"/>
+    <col width="20" customWidth="1" min="44" max="44"/>
+    <col width="20" customWidth="1" min="45" max="45"/>
+    <col width="20" customWidth="1" min="46" max="46"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="48" max="48"/>
+    <col width="20" customWidth="1" min="49" max="49"/>
+    <col width="20" customWidth="1" min="50" max="50"/>
+    <col width="20" customWidth="1" min="51" max="51"/>
+    <col width="20" customWidth="1" min="52" max="52"/>
+    <col width="20" customWidth="1" min="53" max="53"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
           <t>VYVOD</t>
         </is>
       </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>OV_tz</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>OV_dtm</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>OV_dto</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>OV_rd</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>NaSign_dtm</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>NaSign_dto</t>
+        </is>
+      </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>OV_tovctoc</t>
+          <t>NaSign_rd</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>OV_hvptoc1_tovctoc</t>
+          <t>srabKontOtkl_m</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>NaOtkl_tovctoc</t>
+          <t>srabKontSign_m</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>OV_ptoc1_tovctoc</t>
+          <t>srabKontOtkl_o</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>OV_ptoc2_tovctoc</t>
+          <t>srabKontSign_o</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>OV_ptoc1_lvarctoc</t>
+          <t>srabKontOtkl_rd</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>OV_ptoc1_ltcblktoc</t>
+          <t>srabKI_m</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>OV_strpalc</t>
+          <t>srabKI_o</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>OV_hvptoc1_strpalc</t>
+          <t>srabKI_rd</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>OV_lvptoc1_strpalc</t>
+          <t>Sbros</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>OV_lvptoc2_strpalc</t>
+          <t>OV_ts</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>OV_tpalc</t>
+          <t>OV_pk</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>OV_hvptoc1_tpalc</t>
+          <t>OV_ok</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>OV_lvptoc1_tpalc</t>
+          <t>OV_lev</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>OV_lvptoc2_tpalc</t>
+          <t>NaSign_pk</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>OV_eqpalc</t>
+          <t>NaSign_ok</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>NaSign_eqpalc</t>
+          <t>NaSign_lev</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
+          <t>srabKontOtkl_pk</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>srabKontOtkl_ok</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>srabKontOtkl_lev</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>OV_ptrc1_talmgaslgc</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>NaOtkl_ptrc1_talmgaslgc</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>srabKont_ptrc1_talmgaslgc</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>srabKI_ptrc1_talmgaslgc</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>OV_ptrc1_ttrgaslgc</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>NaSign_ptrc1_ttrgaslgc</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>srabKont_ptrc1_ttrgaslgc</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>srabKI_ptrc1_ttrgaslgc</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>OV_ptrc1_tltcgaslgc</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>NaSign_ptrc1_tltcgaslgc</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>srabKont_ptrc1_tltcgaslgc</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>srabKI_ptrc1_tltcgaslgc</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>OV_tprmofflvlgc</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>OV_ptrc1_tprmofflvlgc</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>OV_rbre1_tprmofflvlgc</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>oil_t_hi_level</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>oil_ltc_hi_level</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>oil_ltc_lo_level</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>oil_ltc_lo_temp</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
           <t>otkaz_so</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>t_masla_zpo</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>OV_tprmofflvlgc</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>OV_ptrc1_tprmofflvlgc</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>OV_rbre1_tprmofflvlgc</t>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>neisp_so</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>vnesh_otk_zdz1</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>vnesh_otk_zdz2</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>vnesh_otk_urov1</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>vnesh_otk_urov2</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>vnesh_otkl_so</t>
         </is>
       </c>
     </row>
@@ -1048,6 +1309,78 @@
         <v>0</v>
       </c>
       <c r="AC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1062,7 +1395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BP2"/>
+  <dimension ref="A1:BM2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1130,348 +1463,330 @@
     <col width="20" customWidth="1" min="63" max="63"/>
     <col width="20" customWidth="1" min="64" max="64"/>
     <col width="20" customWidth="1" min="65" max="65"/>
-    <col width="20" customWidth="1" min="66" max="66"/>
-    <col width="20" customWidth="1" min="67" max="67"/>
-    <col width="20" customWidth="1" min="68" max="68"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>vvod_hvptoc1_tovctoc</t>
+          <t>vvod_oilptrc1_apttechlgc</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>oper_vyvod_hvptoc1_tovctoc</t>
+          <t>oper_vyvod_oilptrc1_apttechlgc</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>pusk_hvptoc1_tovctoc</t>
+          <t>srab_oilptrc1_apttechlgc</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>io_hvptoc1_tovctoc</t>
+          <t>srabsign_oilptrc1_apttechlgc</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>srab_hvptoc1_tovctoc</t>
+          <t>zablok_oilptrc1_apttechlgc</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>srabotkl_hvptoc1_tovctoc</t>
+          <t>vvod_winptrc1_apttechlgc</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>vvod_ptoc1_tovctoc</t>
+          <t>oper_vyvod_winptrc1_apttechlgc</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>oper_vyvod_ptoc1_tovctoc</t>
+          <t>srab_winptrc1_apttechlgc</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>pusk_ptoc1_tovctoc</t>
+          <t>srabsign_winptrc1_apttechlgc</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>io_ptoc1_tovctoc</t>
+          <t>zablok_winptrc1_apttechlgc</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>srab_ptoc1_tovctoc</t>
+          <t>vvod_vlvptrc1_apttechlgc</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>srabotkl_ptoc1_tovctoc</t>
+          <t>oper_vyvod_vlvptrc1_apttechlgc</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>vvod_ptoc2_tovctoc</t>
+          <t>srab_vlvptrc1_apttechlgc</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>oper_vyvod_ptoc2_tovctoc</t>
+          <t>srabsign_vlvptrc1_apttechlgc</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>pusk_ptoc2_tovctoc</t>
+          <t>zablok_vlvptrc1_apttechlgc</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>io_ptoc2_tovctoc</t>
+          <t>vvod_prvlvptrc1_almtechlgc</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>srab_ptoc2_tovctoc</t>
+          <t>oper_vyvod_prvlvptrc1_almtechlgc</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>srabotkl_ptoc2_tovctoc</t>
+          <t>srab_prvlvptrc1_almtechlgc</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>srab_tovctoc</t>
+          <t>srabsign_prvlvptrc1_almtechlgc</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>vvod_ptoc1_lvarctoc</t>
+          <t>vvod_shvlvptrc1_almtechlgc</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>oper_vyvod_ptoc1_lvarctoc</t>
+          <t>oper_vyvod_shvlvptrc1_almtechlgc</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>pusk_ptoc1_lvarctoc</t>
+          <t>srab_shvlvptrc1_almtechlgc</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>io_ptoc1_lvarctoc</t>
+          <t>srabsign_shvlvptrc1_almtechlgc</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>vvod_ptoc1_ltcblktoc</t>
+          <t>vvod_levptrc1_almtechlgc</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>oper_vyvod_ptoc1_ltcblktoc</t>
+          <t>oper_vyvod_levptrc1_almtechlgc</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>pusk_ptoc1_ltcblktoc</t>
+          <t>srab_levptrc1_almtechlgc</t>
         </is>
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>io_ptoc1_ltcblktoc</t>
+          <t>srabsign_levptrc1_almtechlgc</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
-          <t>vvod_hvptoc1_strpalc</t>
+          <t>vvod_ptrc1_talmgaslgc</t>
         </is>
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
-          <t>oper_vyvod_hvptoc1_strpalc</t>
+          <t>oper_vyvod_ptrc1_talmgaslgc</t>
         </is>
       </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
-          <t>pusk_hvptoc1_strpalc</t>
+          <t>srab_ptrc1_talmgaslgc</t>
         </is>
       </c>
       <c r="AE1" s="1" t="inlineStr">
         <is>
-          <t>io_hvptoc1_strpalc</t>
+          <t>srabsign_ptrc1_talmgaslgc</t>
         </is>
       </c>
       <c r="AF1" s="1" t="inlineStr">
         <is>
-          <t>vvod_lvptoc1_strpalc</t>
+          <t>zablok_ptrc1_talmgaslgc</t>
         </is>
       </c>
       <c r="AG1" s="1" t="inlineStr">
         <is>
-          <t>oper_vyvod_lvptoc1_strpalc</t>
+          <t>vvod_ptrc1_ttrgaslgc</t>
         </is>
       </c>
       <c r="AH1" s="1" t="inlineStr">
         <is>
-          <t>pusk_lvptoc1_strpalc</t>
+          <t>oper_vyvod_ptrc1_ttrgaslgc</t>
         </is>
       </c>
       <c r="AI1" s="1" t="inlineStr">
         <is>
-          <t>io_lvptoc1_strpalc</t>
+          <t>srab_ptrc1_ttrgaslgc</t>
         </is>
       </c>
       <c r="AJ1" s="1" t="inlineStr">
         <is>
-          <t>vvod_lvptoc2_strpalc</t>
+          <t>srabsign_ptrc1_ttrgaslgc</t>
         </is>
       </c>
       <c r="AK1" s="1" t="inlineStr">
         <is>
-          <t>oper_vyvod_lvptoc2_strpalc</t>
+          <t>zablok_ptrc1_ttrgaslgc</t>
         </is>
       </c>
       <c r="AL1" s="1" t="inlineStr">
         <is>
-          <t>pusk_lvptoc2_strpalc</t>
+          <t>vvod_ptrc1_tltcgaslgc</t>
         </is>
       </c>
       <c r="AM1" s="1" t="inlineStr">
         <is>
-          <t>io_lvptoc2_strpalc</t>
+          <t>oper_vyvod_ptrc1_tltcgaslgc</t>
         </is>
       </c>
       <c r="AN1" s="1" t="inlineStr">
         <is>
-          <t>pusk_strpalc</t>
+          <t>srab_ptrc1_tltcgaslgc</t>
         </is>
       </c>
       <c r="AO1" s="1" t="inlineStr">
         <is>
-          <t>vvod_strpalc</t>
+          <t>srabsign_ptrc1_tltcgaslgc</t>
         </is>
       </c>
       <c r="AP1" s="1" t="inlineStr">
         <is>
-          <t>vvod_hvptoc1_tpalc</t>
+          <t>zablok_ptrc1_tltcgaslgc</t>
         </is>
       </c>
       <c r="AQ1" s="1" t="inlineStr">
         <is>
-          <t>oper_vyvod_hvptoc1_tpalc</t>
+          <t>vvod_ptrc1_tprmofflvlgc</t>
         </is>
       </c>
       <c r="AR1" s="1" t="inlineStr">
         <is>
-          <t>pusk_hvptoc1_tpalc</t>
+          <t>oper_vyvod_ptrc1_tprmofflvlgc</t>
         </is>
       </c>
       <c r="AS1" s="1" t="inlineStr">
         <is>
-          <t>io_hvptoc1_tpalc</t>
+          <t>pusk_ptrc1_tprmofflvlgc</t>
         </is>
       </c>
       <c r="AT1" s="1" t="inlineStr">
         <is>
-          <t>vvod_lvptoc1_tpalc</t>
+          <t>srab_ptrc1_tprmofflvlgc</t>
         </is>
       </c>
       <c r="AU1" s="1" t="inlineStr">
         <is>
-          <t>oper_vyvod_lvptoc1_tpalc</t>
+          <t>vvod_rbre1_tprmofflvlgc</t>
         </is>
       </c>
       <c r="AV1" s="1" t="inlineStr">
         <is>
-          <t>pusk_lvptoc1_tpalc</t>
+          <t>oper_vyvod_rbre1_tprmofflvlgc</t>
         </is>
       </c>
       <c r="AW1" s="1" t="inlineStr">
         <is>
-          <t>io_lvptoc1_tpalc</t>
+          <t>zapret_rbre1_tprmofflvlgc</t>
         </is>
       </c>
       <c r="AX1" s="1" t="inlineStr">
         <is>
-          <t>vvod_lvptoc2_tpalc</t>
+          <t>SS_gz_sign</t>
         </is>
       </c>
       <c r="AY1" s="1" t="inlineStr">
         <is>
-          <t>oper_vyvod_lvptoc2_tpalc</t>
+          <t>SS_gz_nizk_isol</t>
         </is>
       </c>
       <c r="AZ1" s="1" t="inlineStr">
         <is>
-          <t>pusk_lvptoc2_tpalc</t>
+          <t>SS_gz_zablok</t>
         </is>
       </c>
       <c r="BA1" s="1" t="inlineStr">
         <is>
-          <t>io_lvptoc2_tpalc</t>
+          <t>SS_tz_sign</t>
         </is>
       </c>
       <c r="BB1" s="1" t="inlineStr">
         <is>
-          <t>pusk_tpalc</t>
+          <t>SS_tz_nizk_isol</t>
         </is>
       </c>
       <c r="BC1" s="1" t="inlineStr">
         <is>
-          <t>vvod_tpalc</t>
+          <t>SS_tz_zablok</t>
         </is>
       </c>
       <c r="BD1" s="1" t="inlineStr">
         <is>
-          <t>vvod_lvoileqpalc_eqpalc</t>
+          <t>SS_ts_sign</t>
         </is>
       </c>
       <c r="BE1" s="1" t="inlineStr">
         <is>
-          <t>oper_vyvod_lvoileqpalc_eqpalc</t>
+          <t>SS_vnesh_otkl</t>
         </is>
       </c>
       <c r="BF1" s="1" t="inlineStr">
         <is>
-          <t>pusk_lvoileqpalc_eqpalc</t>
+          <t>SS_vyh_zepi_razobr</t>
         </is>
       </c>
       <c r="BG1" s="1" t="inlineStr">
         <is>
-          <t>srabsign_lvoileqpalc_eqpalc</t>
+          <t>SS_bi_vyved</t>
         </is>
       </c>
       <c r="BH1" s="1" t="inlineStr">
         <is>
-          <t>srab_lvoileqpalc_eqpalc</t>
+          <t>SS_ot_sign</t>
         </is>
       </c>
       <c r="BI1" s="1" t="inlineStr">
         <is>
-          <t>vvod_ptrc1_tprmofflvlgc</t>
+          <t>SS_neispr_ot_gz</t>
         </is>
       </c>
       <c r="BJ1" s="1" t="inlineStr">
         <is>
-          <t>oper_vyvod_ptrc1_tprmofflvlgc</t>
+          <t>SS_neispr_ot_tz</t>
         </is>
       </c>
       <c r="BK1" s="1" t="inlineStr">
         <is>
-          <t>pusk_ptrc1_tprmofflvlgc</t>
+          <t>SS_ot_nn_sign</t>
         </is>
       </c>
       <c r="BL1" s="1" t="inlineStr">
         <is>
-          <t>srab_ptrc1_tprmofflvlgc</t>
+          <t>SS_obsh_vnesh_sign</t>
         </is>
       </c>
       <c r="BM1" s="1" t="inlineStr">
-        <is>
-          <t>vvod_rbre1_tprmofflvlgc</t>
-        </is>
-      </c>
-      <c r="BN1" s="1" t="inlineStr">
-        <is>
-          <t>oper_vyvod_rbre1_tprmofflvlgc</t>
-        </is>
-      </c>
-      <c r="BO1" s="1" t="inlineStr">
-        <is>
-          <t>zapret_rbre1_tprmofflvlgc</t>
-        </is>
-      </c>
-      <c r="BP1" s="1" t="inlineStr">
         <is>
           <t>pusk_lvalh</t>
         </is>
@@ -1688,9 +2003,9 @@
           <t>0</t>
         </is>
       </c>
-      <c r="AQ2" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="AQ2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
       <c r="AR2" t="inlineStr">
@@ -1708,9 +2023,9 @@
           <t>0</t>
         </is>
       </c>
-      <c r="AU2" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="AU2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
       <c r="AV2" t="inlineStr">
@@ -1778,9 +2093,9 @@
           <t>0</t>
         </is>
       </c>
-      <c r="BI2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
+      <c r="BI2" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
       <c r="BJ2" t="inlineStr">
@@ -1798,22 +2113,7 @@
           <t>0</t>
         </is>
       </c>
-      <c r="BM2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BN2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="BO2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="BP2" t="inlineStr">
+      <c r="BM2" t="inlineStr">
         <is>
           <t>0</t>
         </is>

</xml_diff>